<commit_message>
add grammar 9 10
</commit_message>
<xml_diff>
--- a/GRAMMAR/10_17_12.xlsx
+++ b/GRAMMAR/10_17_12.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\N2_2025_12\GRAMMAR\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73D77D28-A693-44D2-A4FC-CC4D177231C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{561AD893-05A3-4C5D-A7CA-529DF52E9A00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12300" yWindow="915" windowWidth="27840" windowHeight="20040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19140" yWindow="1005" windowWidth="19260" windowHeight="19995" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="92">
   <si>
     <t>Fre</t>
   </si>
@@ -30,9 +30,6 @@
     <t>文法</t>
   </si>
   <si>
-    <t>含义</t>
-  </si>
-  <si>
     <t>读音</t>
   </si>
   <si>
@@ -288,6 +285,117 @@
   </si>
   <si>
     <t>原形"いたす","する"自谦</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>疑问词+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>かというと</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>要说为什么…</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>たばかり</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>刚刚(主观)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ということだ</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>传闻</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>というものだ</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>也就是…</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>おります</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>「いる」自谦语</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ございます</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>あります 郑重语</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>どうやって＋…＋か</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>如何…呢？</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>～通り</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>按照</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>わりに</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>与…相比(转折)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>なめらか</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>光滑；顺利；流畅</t>
+  </si>
+  <si>
+    <t>光滑；顺利；流畅</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>単に</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>仅仅；只不过</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>〜らしいです</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>好像</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -295,7 +403,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -325,6 +433,20 @@
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Yu Gothic"/>
+      <family val="3"/>
+      <charset val="128"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFBDB7AE"/>
+      <name val="黑体"/>
+      <family val="3"/>
+      <charset val="134"/>
     </font>
   </fonts>
   <fills count="2">
@@ -362,7 +484,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -370,6 +492,10 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -672,7 +798,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="9" style="2" customWidth="1"/>
@@ -683,21 +809,21 @@
     <col min="6" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:5" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.15">
@@ -705,10 +831,10 @@
         <v>0</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>5</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.15">
@@ -716,10 +842,10 @@
         <v>0</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>7</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.15">
@@ -727,13 +853,13 @@
         <v>0</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>10</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.15">
@@ -741,10 +867,10 @@
         <v>0</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>12</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.15">
@@ -752,10 +878,10 @@
         <v>0</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>14</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.15">
@@ -763,10 +889,10 @@
         <v>0</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>16</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.15">
@@ -774,13 +900,13 @@
         <v>0</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="E8" s="2" t="s">
         <v>19</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.15">
@@ -788,10 +914,10 @@
         <v>0</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>21</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.15">
@@ -799,10 +925,10 @@
         <v>0</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>23</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.15">
@@ -810,13 +936,13 @@
         <v>0</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.15">
@@ -824,10 +950,10 @@
         <v>0</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>26</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.15">
@@ -835,10 +961,10 @@
         <v>0</v>
       </c>
       <c r="B13" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>28</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.15">
@@ -846,10 +972,10 @@
         <v>0</v>
       </c>
       <c r="B14" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>30</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.15">
@@ -857,10 +983,10 @@
         <v>0</v>
       </c>
       <c r="B15" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>32</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.15">
@@ -868,10 +994,10 @@
         <v>0</v>
       </c>
       <c r="B16" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>34</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.15">
@@ -879,10 +1005,10 @@
         <v>0</v>
       </c>
       <c r="B17" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>36</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.15">
@@ -890,13 +1016,13 @@
         <v>0</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.15">
@@ -904,13 +1030,13 @@
         <v>0</v>
       </c>
       <c r="B19" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="E19" s="2" t="s">
         <v>40</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.15">
@@ -918,10 +1044,10 @@
         <v>0</v>
       </c>
       <c r="B20" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>42</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.15">
@@ -929,10 +1055,10 @@
         <v>0</v>
       </c>
       <c r="B21" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C21" s="2" t="s">
         <v>44</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.15">
@@ -940,10 +1066,10 @@
         <v>0</v>
       </c>
       <c r="B22" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C22" s="2" t="s">
         <v>46</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.15">
@@ -951,10 +1077,10 @@
         <v>0</v>
       </c>
       <c r="B23" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>48</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.15">
@@ -962,10 +1088,10 @@
         <v>0</v>
       </c>
       <c r="B24" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C24" s="2" t="s">
         <v>50</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.15">
@@ -973,10 +1099,10 @@
         <v>0</v>
       </c>
       <c r="B25" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C25" s="2" t="s">
         <v>52</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.15">
@@ -984,10 +1110,10 @@
         <v>0</v>
       </c>
       <c r="B26" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C26" s="2" t="s">
         <v>54</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.15">
@@ -995,10 +1121,10 @@
         <v>0</v>
       </c>
       <c r="B27" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C27" s="2" t="s">
         <v>56</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.15">
@@ -1006,10 +1132,10 @@
         <v>0</v>
       </c>
       <c r="B28" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C28" s="2" t="s">
         <v>58</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.15">
@@ -1017,10 +1143,10 @@
         <v>0</v>
       </c>
       <c r="B29" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C29" s="2" t="s">
         <v>60</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.15">
@@ -1028,10 +1154,142 @@
         <v>0</v>
       </c>
       <c r="B30" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C30" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="C30" s="2" t="s">
-        <v>63</v>
+    </row>
+    <row r="31" spans="1:5" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A31" s="2">
+        <v>1</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A32" s="2">
+        <v>1</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A33" s="2">
+        <v>1</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A34" s="2">
+        <v>1</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A35" s="2">
+        <v>1</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A36" s="2">
+        <v>1</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A37" s="2">
+        <v>1</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A38" s="2">
+        <v>1</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A39" s="2">
+        <v>1</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A40" s="2">
+        <v>1</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A41" s="2">
+        <v>1</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.15">
+      <c r="A42" s="2">
+        <v>1</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>91</v>
       </c>
     </row>
   </sheetData>

</xml_diff>